<commit_message>
added updated data set to the code
</commit_message>
<xml_diff>
--- a/flight_ticket booking/tickets.xlsx
+++ b/flight_ticket booking/tickets.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -991,10 +991,8 @@
           <t>karthik</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>789789789789</t>
-        </is>
+      <c r="E11" t="n">
+        <v>789789789789</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1024,6 +1022,171 @@
       <c r="M11" t="inlineStr">
         <is>
           <t>Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>8978344990</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Biju Patnaik International Airport (BBI)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Jaipur International Airport (JAI)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>karthik</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>789456258741</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>5495</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>25</v>
+      </c>
+      <c r="J12" t="n">
+        <v>15</v>
+      </c>
+      <c r="K12" t="n">
+        <v>5535</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>10-May-2026 07:11 PM</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>8978344990</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Biju Patnaik International Airport (BBI)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Jaipur International Airport (JAI)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>vamshi</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>963258741321</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>5495</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>25</v>
+      </c>
+      <c r="J13" t="n">
+        <v>15</v>
+      </c>
+      <c r="K13" t="n">
+        <v>5535</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>10-May-2026 07:11 PM</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>8978344990</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Biju Patnaik International Airport (BBI)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Jaipur International Airport (JAI)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>raju</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>852963741852</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>5495</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>25</v>
+      </c>
+      <c r="J14" t="n">
+        <v>15</v>
+      </c>
+      <c r="K14" t="n">
+        <v>5535</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>10-May-2026 07:11 PM</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>UPI</t>
         </is>
       </c>
     </row>

</xml_diff>